<commit_message>
Add v2 personal-distribution features: swappable scene vocab, storage, search
- Simple Excel template v2 (10 columns: maker, TAIS code, specs added)
- Editable scene/concern vocab sheet; navi and filters follow imported vocab
- Persist imported catalog in localStorage with restore on startup
- Full CSV template v2 (16 columns with taisCode)
- Product name/maker/TAIS search page, scene filter in genre lists
- Auto similar-products section on detail page
- Docs and in-app wording updated for personal use distribution

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/products-template-simple.xlsx
+++ b/public/products-template-simple.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="商品リスト" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="選択肢" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="シーン設定" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="選択肢" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -56,9 +57,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,16 +428,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -444,30 +451,45 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>メーカー</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>分類</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>価格(円)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>TAISコード</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ひとこと説明</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>仕様</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>困りごと1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>困りごと2</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>誰が使う</t>
         </is>
@@ -481,28 +503,44 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>あおぞら福祉機器</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>歩行補助</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>1200</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>01234-000001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>軽くてにぎりやすい定番の一本杖</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>重さ:290g
+高さ調節:71〜94cm(10段階)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>ふらつく・転びやすい</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>屋外の外出が不安</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>本人が使う</t>
         </is>
@@ -514,30 +552,38 @@
           <t>ささえ四点杖ワイド</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
         <is>
           <t>歩行補助</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>1800</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
         <is>
           <t>自立するから立ち上がり時も支えになる四点杖</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>重さ:640g
+高さ調節:66〜89cm</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>ふらつく・転びやすい</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>支えがないと立てない</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>本人が使う</t>
         </is>
@@ -551,28 +597,35 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>みらいケア</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>見守り・生活サポート</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>2000</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
         <is>
           <t>夜中の動きをやさしく知らせる見守りセンサー</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
         <is>
           <t>夜中に動き回る</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>一人にするのが心配</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>どちらも</t>
         </is>
@@ -580,14 +633,14 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="C2:C1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>'選択肢'!$A$2:$A$10</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E1001 F2:F1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>'選択肢'!$B$2:$B$32</formula1>
+    <dataValidation sqref="H2:H1001 I2:I1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>'シーン設定'!$B$2:$B$121</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>'選択肢'!$C$2:$C$4</formula1>
+    <dataValidation sqref="J2:J1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>'選択肢'!$B$2:$B$4</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -600,7 +653,409 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:B32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>場面</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>困りごと</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>歩く・移動</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ふらつく・転びやすい</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>歩く・移動</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>長い距離を歩けない</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>歩く・移動</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>屋外の外出が不安</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>歩く・移動</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>段差につまずく</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>歩く・移動</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>荷物を持って歩けない</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>立つ・座る</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>立ち上がるのがつらい</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>立つ・座る</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>座るときにドスンと落ちる</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>立つ・座る</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ひざ・腰が痛い</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>立つ・座る</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>支えがないと立てない</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>寝る・起きる</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>起き上がれない</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>寝る・起きる</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ベッドから立ち上がれない</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>寝る・起きる</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>寝返りが打てない</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>寝る・起きる</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>床ずれが心配</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>寝る・起きる</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>布団の上げ下ろしがつらい</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>お風呂</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>浴槽をまたぐのがこわい</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>お風呂</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>浴室で立ち上がれない</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>お風呂</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>滑るのが心配</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>お風呂</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>体を洗いにくい</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>お風呂</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>浴室まで移動できない</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>トイレ</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>トイレまで間に合わない</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>トイレ</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>便座から立ち上がれない</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>トイレ</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>夜のトイレが不安</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>トイレ</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>トイレまで移動できない</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>食事</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>箸・スプーンが持ちにくい</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>食事</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>食器が滑る・こぼす</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>食事</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>姿勢を保てない</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>食事</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>飲み込みが心配</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>見守り・その他</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>一人にするのが心配</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>見守り・その他</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>夜中に動き回る</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>見守り・その他</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>呼ばれてもすぐ行けない</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>見守り・その他</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>介助者の負担が大きい</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -611,11 +1066,6 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>困りごと</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
           <t>誰が使う</t>
         </is>
       </c>
@@ -628,11 +1078,6 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ふらつく・転びやすい</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
           <t>本人が使う</t>
         </is>
       </c>
@@ -645,11 +1090,6 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>長い距離を歩けない</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
           <t>家族の介護に使う</t>
         </is>
       </c>
@@ -662,11 +1102,6 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>屋外の外出が不安</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
           <t>どちらも</t>
         </is>
       </c>
@@ -677,11 +1112,6 @@
           <t>床ずれ予防・マットレス</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>段差につまずく</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -689,11 +1119,6 @@
           <t>移乗・移動サポート</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>荷物を持って歩けない</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -701,11 +1126,6 @@
           <t>入浴</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>立ち上がるのがつらい</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -713,11 +1133,6 @@
           <t>トイレ・排泄</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>座るときにドスンと落ちる</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -725,175 +1140,11 @@
           <t>手すり・スロープ・段差</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>ひざ・腰が痛い</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
           <t>見守り・生活サポート</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>支えがないと立てない</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>起き上がれない</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>ベッドから立ち上がれない</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>寝返りが打てない</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>床ずれが心配</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>布団の上げ下ろしがつらい</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>浴槽をまたぐのがこわい</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>浴室で立ち上がれない</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>滑るのが心配</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>体を洗いにくい</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>浴室まで移動できない</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>トイレまで間に合わない</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>便座から立ち上がれない</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>夜のトイレが不安</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>トイレまで移動できない</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>箸・スプーンが持ちにくい</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>食器が滑る・こぼす</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>姿勢を保てない</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>飲み込みが心配</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>一人にするのが心配</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>夜中に動き回る</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>呼ばれてもすぐ行けない</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>介助者の負担が大きい</t>
         </is>
       </c>
     </row>

</xml_diff>